<commit_message>
CCTP-13594 add csv validation for phoneNumberDialed and greeting
</commit_message>
<xml_diff>
--- a/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/Legacy-Comparion.xlsx
+++ b/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/Legacy-Comparion.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n0354604\IdeaProjects\cicct-softphone-admin-ui-merge-refactor\src\components\tabs\dynamicCallFlow\phoneNumber\Xlsx\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/CaseSensitive/cicct-softphone-admin-ui/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E38B82C-326F-47D6-9C0C-AB6C057E2C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EB08942-B5F4-5641-9D13-5275017615F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="call-flow-1718140016159" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1350" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1448" uniqueCount="396">
   <si>
     <t>dialedPhoneNumber</t>
   </si>
@@ -914,6 +927,300 @@
   </si>
   <si>
     <t>2023-06-13T17:56:48.510Z</t>
+  </si>
+  <si>
+    <t>+19374381966</t>
+  </si>
+  <si>
+    <t>+18045273902</t>
+  </si>
+  <si>
+    <t>+12074822171</t>
+  </si>
+  <si>
+    <t>+12012217220</t>
+  </si>
+  <si>
+    <t>+18663764517</t>
+  </si>
+  <si>
+    <t>+19256590416</t>
+  </si>
+  <si>
+    <t>+16102055988</t>
+  </si>
+  <si>
+    <t>+13012625242</t>
+  </si>
+  <si>
+    <t>+15182431128</t>
+  </si>
+  <si>
+    <t>+18446468596</t>
+  </si>
+  <si>
+    <t>+18594880750</t>
+  </si>
+  <si>
+    <t>+17044965966</t>
+  </si>
+  <si>
+    <t>+15595128319</t>
+  </si>
+  <si>
+    <t>+19096871073</t>
+  </si>
+  <si>
+    <t>+16784033612</t>
+  </si>
+  <si>
+    <t>+17706883859</t>
+  </si>
+  <si>
+    <t>+14402641163</t>
+  </si>
+  <si>
+    <t>+17815560159</t>
+  </si>
+  <si>
+    <t>+16319288591</t>
+  </si>
+  <si>
+    <t>+18442848580</t>
+  </si>
+  <si>
+    <t>+11165122067</t>
+  </si>
+  <si>
+    <t>+16105689457</t>
+  </si>
+  <si>
+    <t>+18442872899</t>
+  </si>
+  <si>
+    <t>+19253929330</t>
+  </si>
+  <si>
+    <t>+11165122305</t>
+  </si>
+  <si>
+    <t>+19527695954</t>
+  </si>
+  <si>
+    <t>+18039084300</t>
+  </si>
+  <si>
+    <t>+16466821422</t>
+  </si>
+  <si>
+    <t>+18039084304</t>
+  </si>
+  <si>
+    <t>+16033385062</t>
+  </si>
+  <si>
+    <t>+18002488320</t>
+  </si>
+  <si>
+    <t>+15053554824</t>
+  </si>
+  <si>
+    <t>+17814712390</t>
+  </si>
+  <si>
+    <t>+18885040156</t>
+  </si>
+  <si>
+    <t>+18882941543</t>
+  </si>
+  <si>
+    <t>+19522295689</t>
+  </si>
+  <si>
+    <t>+19012159840</t>
+  </si>
+  <si>
+    <t>+13037230365</t>
+  </si>
+  <si>
+    <t>+12012212270</t>
+  </si>
+  <si>
+    <t>+18475512866</t>
+  </si>
+  <si>
+    <t>+18668712671</t>
+  </si>
+  <si>
+    <t>+14018241106</t>
+  </si>
+  <si>
+    <t>+19012159786</t>
+  </si>
+  <si>
+    <t>+14806064205</t>
+  </si>
+  <si>
+    <t>+15856133090</t>
+  </si>
+  <si>
+    <t>+16126567392</t>
+  </si>
+  <si>
+    <t>+14086781321</t>
+  </si>
+  <si>
+    <t>+18449680236</t>
+  </si>
+  <si>
+    <t>+11165122309</t>
+  </si>
+  <si>
+    <t>+11165122063</t>
+  </si>
+  <si>
+    <t>+16102055991</t>
+  </si>
+  <si>
+    <t>+18448780598</t>
+  </si>
+  <si>
+    <t>+19203434305</t>
+  </si>
+  <si>
+    <t>+15053554827</t>
+  </si>
+  <si>
+    <t>+15053554829</t>
+  </si>
+  <si>
+    <t>+16309194407</t>
+  </si>
+  <si>
+    <t>+18442872862</t>
+  </si>
+  <si>
+    <t>+16023664078</t>
+  </si>
+  <si>
+    <t>+12074806116</t>
+  </si>
+  <si>
+    <t>+18303877926</t>
+  </si>
+  <si>
+    <t>+18582553962</t>
+  </si>
+  <si>
+    <t>+17086753641</t>
+  </si>
+  <si>
+    <t>+18058982637</t>
+  </si>
+  <si>
+    <t>+12059099009</t>
+  </si>
+  <si>
+    <t>+18604947620</t>
+  </si>
+  <si>
+    <t>+14698088704</t>
+  </si>
+  <si>
+    <t>+12122082849</t>
+  </si>
+  <si>
+    <t>+18446210949</t>
+  </si>
+  <si>
+    <t>+16038981747</t>
+  </si>
+  <si>
+    <t>+12704186304</t>
+  </si>
+  <si>
+    <t>+16094037594</t>
+  </si>
+  <si>
+    <t>+18084870628</t>
+  </si>
+  <si>
+    <t>+18005987561</t>
+  </si>
+  <si>
+    <t>+18448591664</t>
+  </si>
+  <si>
+    <t>+18442153023</t>
+  </si>
+  <si>
+    <t>+17704072207</t>
+  </si>
+  <si>
+    <t>+16237071176</t>
+  </si>
+  <si>
+    <t>+11165122202</t>
+  </si>
+  <si>
+    <t>+18447172505</t>
+  </si>
+  <si>
+    <t>+16827858101</t>
+  </si>
+  <si>
+    <t>+18452886684</t>
+  </si>
+  <si>
+    <t>+19086731724</t>
+  </si>
+  <si>
+    <t>+14072043651</t>
+  </si>
+  <si>
+    <t>+11165122318</t>
+  </si>
+  <si>
+    <t>+15086213800</t>
+  </si>
+  <si>
+    <t>+12813924333</t>
+  </si>
+  <si>
+    <t>+12038050236</t>
+  </si>
+  <si>
+    <t>+12068920075</t>
+  </si>
+  <si>
+    <t>+19785393223</t>
+  </si>
+  <si>
+    <t>+14402642930</t>
+  </si>
+  <si>
+    <t>+17044965969</t>
+  </si>
+  <si>
+    <t>+13035680570</t>
+  </si>
+  <si>
+    <t>+18134396643</t>
+  </si>
+  <si>
+    <t>+17192160070</t>
+  </si>
+  <si>
+    <t>+16144582016</t>
+  </si>
+  <si>
+    <t>+17029639622</t>
+  </si>
+  <si>
+    <t>+17043601846</t>
+  </si>
+  <si>
+    <t>+17815651907</t>
   </si>
 </sst>
 </file>
@@ -1776,13 +2083,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AL99"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1898,9 +2205,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>19374381966</v>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>298</v>
       </c>
       <c r="E2" t="s">
         <v>38</v>
@@ -1951,9 +2258,9 @@
         <v>167</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>18045273902</v>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>299</v>
       </c>
       <c r="E3" t="s">
         <v>38</v>
@@ -2004,9 +2311,9 @@
         <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>12074822171</v>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>300</v>
       </c>
       <c r="D4" t="s">
         <v>53</v>
@@ -2063,9 +2370,9 @@
         <v>185</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>12012217220</v>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>301</v>
       </c>
       <c r="E5" t="s">
         <v>38</v>
@@ -2116,9 +2423,9 @@
         <v>187</v>
       </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>18663764517</v>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>302</v>
       </c>
       <c r="E6" t="s">
         <v>38</v>
@@ -2169,9 +2476,9 @@
         <v>191</v>
       </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>19256590416</v>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>303</v>
       </c>
       <c r="D7" t="s">
         <v>68</v>
@@ -2228,9 +2535,9 @@
         <v>202</v>
       </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>16102055988</v>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>304</v>
       </c>
       <c r="D8">
         <v>7015241</v>
@@ -2281,9 +2588,9 @@
         <v>205</v>
       </c>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>13012625242</v>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>305</v>
       </c>
       <c r="E9" t="s">
         <v>38</v>
@@ -2334,9 +2641,9 @@
         <v>206</v>
       </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>15182431128</v>
+    <row r="10" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>306</v>
       </c>
       <c r="E10" t="s">
         <v>38</v>
@@ -2390,9 +2697,9 @@
         <v>213</v>
       </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>18446468596</v>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>307</v>
       </c>
       <c r="E11" t="s">
         <v>38</v>
@@ -2443,9 +2750,9 @@
         <v>216</v>
       </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>18594880750</v>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>308</v>
       </c>
       <c r="D12">
         <v>6153661</v>
@@ -2496,9 +2803,9 @@
         <v>223</v>
       </c>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>17044965966</v>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>309</v>
       </c>
       <c r="E13" t="s">
         <v>38</v>
@@ -2552,9 +2859,9 @@
         <v>232</v>
       </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>15595128319</v>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>310</v>
       </c>
       <c r="D14" t="s">
         <v>87</v>
@@ -2611,9 +2918,9 @@
         <v>241</v>
       </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>19096871073</v>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>311</v>
       </c>
       <c r="D15" t="s">
         <v>90</v>
@@ -2670,9 +2977,9 @@
         <v>248</v>
       </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>16784033612</v>
+    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>312</v>
       </c>
       <c r="D16">
         <v>6158696</v>
@@ -2723,9 +3030,9 @@
         <v>249</v>
       </c>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>17706883859</v>
+    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>313</v>
       </c>
       <c r="E17" t="s">
         <v>38</v>
@@ -2779,9 +3086,9 @@
         <v>258</v>
       </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>14402641163</v>
+    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>314</v>
       </c>
       <c r="E18" t="s">
         <v>38</v>
@@ -2835,9 +3142,9 @@
         <v>264</v>
       </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>17815560159</v>
+    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>315</v>
       </c>
       <c r="E19" t="s">
         <v>38</v>
@@ -2891,9 +3198,9 @@
         <v>273</v>
       </c>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>16319288591</v>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>316</v>
       </c>
       <c r="E20" t="s">
         <v>38</v>
@@ -2941,9 +3248,9 @@
         <v>281</v>
       </c>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>18442848580</v>
+    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>317</v>
       </c>
       <c r="E21" t="s">
         <v>38</v>
@@ -2994,9 +3301,9 @@
         <v>290</v>
       </c>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>11165122067</v>
+    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>318</v>
       </c>
       <c r="E22" t="s">
         <v>38</v>
@@ -3044,9 +3351,9 @@
         <v>308</v>
       </c>
     </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>16105689457</v>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>319</v>
       </c>
       <c r="E23" t="s">
         <v>38</v>
@@ -3100,9 +3407,9 @@
         <v>312</v>
       </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>18442872899</v>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>320</v>
       </c>
       <c r="E24" t="s">
         <v>38</v>
@@ -3153,9 +3460,9 @@
         <v>325</v>
       </c>
     </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>19253929330</v>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>321</v>
       </c>
       <c r="D25" t="s">
         <v>116</v>
@@ -3212,9 +3519,9 @@
         <v>336</v>
       </c>
     </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>11165122305</v>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>322</v>
       </c>
       <c r="E26" t="s">
         <v>38</v>
@@ -3262,9 +3569,9 @@
         <v>343</v>
       </c>
     </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>19527695954</v>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>323</v>
       </c>
       <c r="D27" t="s">
         <v>120</v>
@@ -3321,9 +3628,9 @@
         <v>351</v>
       </c>
     </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>18039084300</v>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>324</v>
       </c>
       <c r="D28">
         <v>6159272</v>
@@ -3374,9 +3681,9 @@
         <v>363</v>
       </c>
     </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>16466821422</v>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>325</v>
       </c>
       <c r="E29" t="s">
         <v>38</v>
@@ -3430,9 +3737,9 @@
         <v>373</v>
       </c>
     </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>18039084304</v>
+    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>326</v>
       </c>
       <c r="E30" t="s">
         <v>38</v>
@@ -3486,9 +3793,9 @@
         <v>377</v>
       </c>
     </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>16033385062</v>
+    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>327</v>
       </c>
       <c r="D31">
         <v>6152421</v>
@@ -3539,9 +3846,9 @@
         <v>387</v>
       </c>
     </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>18002488320</v>
+    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>328</v>
       </c>
       <c r="E32" t="s">
         <v>38</v>
@@ -3592,9 +3899,9 @@
         <v>388</v>
       </c>
     </row>
-    <row r="33" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>15053554824</v>
+    <row r="33" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>329</v>
       </c>
       <c r="D33" t="s">
         <v>133</v>
@@ -3651,9 +3958,9 @@
         <v>398</v>
       </c>
     </row>
-    <row r="34" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>17814712390</v>
+    <row r="34" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>330</v>
       </c>
       <c r="E34" t="s">
         <v>38</v>
@@ -3707,9 +4014,9 @@
         <v>420</v>
       </c>
     </row>
-    <row r="35" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>18885040156</v>
+    <row r="35" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>331</v>
       </c>
       <c r="E35" t="s">
         <v>38</v>
@@ -3757,9 +4064,9 @@
         <v>422</v>
       </c>
     </row>
-    <row r="36" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>18882941543</v>
+    <row r="36" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>332</v>
       </c>
       <c r="E36" t="s">
         <v>38</v>
@@ -3807,9 +4114,9 @@
         <v>423</v>
       </c>
     </row>
-    <row r="37" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>19522295689</v>
+    <row r="37" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>333</v>
       </c>
       <c r="D37" t="s">
         <v>143</v>
@@ -3866,9 +4173,9 @@
         <v>425</v>
       </c>
     </row>
-    <row r="38" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>19012159840</v>
+    <row r="38" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>334</v>
       </c>
       <c r="E38" t="s">
         <v>38</v>
@@ -3922,9 +4229,9 @@
         <v>432</v>
       </c>
     </row>
-    <row r="39" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>13037230365</v>
+    <row r="39" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>335</v>
       </c>
       <c r="D39" t="s">
         <v>149</v>
@@ -3981,9 +4288,9 @@
         <v>460</v>
       </c>
     </row>
-    <row r="40" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>12012212270</v>
+    <row r="40" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>336</v>
       </c>
       <c r="E40" t="s">
         <v>38</v>
@@ -4031,9 +4338,9 @@
         <v>468</v>
       </c>
     </row>
-    <row r="41" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>18475512866</v>
+    <row r="41" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>337</v>
       </c>
       <c r="D41" t="s">
         <v>154</v>
@@ -4090,9 +4397,9 @@
         <v>501</v>
       </c>
     </row>
-    <row r="42" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>18668712671</v>
+    <row r="42" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>338</v>
       </c>
       <c r="E42" t="s">
         <v>38</v>
@@ -4143,9 +4450,9 @@
         <v>537</v>
       </c>
     </row>
-    <row r="43" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>14018241106</v>
+    <row r="43" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>339</v>
       </c>
       <c r="E43" t="s">
         <v>38</v>
@@ -4199,9 +4506,9 @@
         <v>542</v>
       </c>
     </row>
-    <row r="44" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>19012159786</v>
+    <row r="44" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>340</v>
       </c>
       <c r="E44" t="s">
         <v>38</v>
@@ -4255,9 +4562,9 @@
         <v>545</v>
       </c>
     </row>
-    <row r="45" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>14806064205</v>
+    <row r="45" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>341</v>
       </c>
       <c r="D45">
         <v>6158015</v>
@@ -4308,9 +4615,9 @@
         <v>547</v>
       </c>
     </row>
-    <row r="46" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>15856133090</v>
+    <row r="46" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>342</v>
       </c>
       <c r="E46" t="s">
         <v>38</v>
@@ -4364,9 +4671,9 @@
         <v>548</v>
       </c>
     </row>
-    <row r="47" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <v>16126567392</v>
+    <row r="47" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>343</v>
       </c>
       <c r="D47">
         <v>6158122</v>
@@ -4417,9 +4724,9 @@
         <v>558</v>
       </c>
     </row>
-    <row r="48" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>14086781321</v>
+    <row r="48" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>344</v>
       </c>
       <c r="D48" t="s">
         <v>171</v>
@@ -4476,9 +4783,9 @@
         <v>561</v>
       </c>
     </row>
-    <row r="49" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>18449680236</v>
+    <row r="49" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>345</v>
       </c>
       <c r="E49" t="s">
         <v>38</v>
@@ -4532,9 +4839,9 @@
         <v>567</v>
       </c>
     </row>
-    <row r="50" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>11165122309</v>
+    <row r="50" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>346</v>
       </c>
       <c r="E50" t="s">
         <v>38</v>
@@ -4582,9 +4889,9 @@
         <v>587</v>
       </c>
     </row>
-    <row r="51" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>11165122063</v>
+    <row r="51" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>347</v>
       </c>
       <c r="E51" t="s">
         <v>38</v>
@@ -4632,9 +4939,9 @@
         <v>599</v>
       </c>
     </row>
-    <row r="52" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>16102055991</v>
+    <row r="52" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>348</v>
       </c>
       <c r="E52" t="s">
         <v>38</v>
@@ -4688,9 +4995,9 @@
         <v>602</v>
       </c>
     </row>
-    <row r="53" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A53">
-        <v>18448780598</v>
+    <row r="53" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>349</v>
       </c>
       <c r="E53" t="s">
         <v>38</v>
@@ -4741,9 +5048,9 @@
         <v>607</v>
       </c>
     </row>
-    <row r="54" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>19203434305</v>
+    <row r="54" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>350</v>
       </c>
       <c r="D54" t="s">
         <v>187</v>
@@ -4800,9 +5107,9 @@
         <v>608</v>
       </c>
     </row>
-    <row r="55" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>15053554827</v>
+    <row r="55" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>351</v>
       </c>
       <c r="D55" t="s">
         <v>190</v>
@@ -4859,9 +5166,9 @@
         <v>612</v>
       </c>
     </row>
-    <row r="56" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>15053554829</v>
+    <row r="56" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>352</v>
       </c>
       <c r="D56" t="s">
         <v>192</v>
@@ -4918,9 +5225,9 @@
         <v>618</v>
       </c>
     </row>
-    <row r="57" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A57">
-        <v>16309194407</v>
+    <row r="57" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>353</v>
       </c>
       <c r="D57" t="s">
         <v>194</v>
@@ -4977,9 +5284,9 @@
         <v>619</v>
       </c>
     </row>
-    <row r="58" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A58">
-        <v>18442872862</v>
+    <row r="58" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>354</v>
       </c>
       <c r="E58" t="s">
         <v>38</v>
@@ -5030,9 +5337,9 @@
         <v>652</v>
       </c>
     </row>
-    <row r="59" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A59">
-        <v>16023664078</v>
+    <row r="59" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>355</v>
       </c>
       <c r="D59" t="s">
         <v>200</v>
@@ -5089,9 +5396,9 @@
         <v>654</v>
       </c>
     </row>
-    <row r="60" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A60">
-        <v>12074806116</v>
+    <row r="60" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>356</v>
       </c>
       <c r="D60">
         <v>6150003</v>
@@ -5142,9 +5449,9 @@
         <v>684</v>
       </c>
     </row>
-    <row r="61" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A61">
-        <v>18303877926</v>
+    <row r="61" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>357</v>
       </c>
       <c r="D61">
         <v>7159155</v>
@@ -5195,9 +5502,9 @@
         <v>687</v>
       </c>
     </row>
-    <row r="62" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A62">
-        <v>18582553962</v>
+    <row r="62" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>358</v>
       </c>
       <c r="D62" t="s">
         <v>205</v>
@@ -5254,9 +5561,9 @@
         <v>705</v>
       </c>
     </row>
-    <row r="63" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A63">
-        <v>17086753641</v>
+    <row r="63" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>359</v>
       </c>
       <c r="D63" t="s">
         <v>208</v>
@@ -5313,9 +5620,9 @@
         <v>747</v>
       </c>
     </row>
-    <row r="64" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A64">
-        <v>18058982637</v>
+    <row r="64" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>360</v>
       </c>
       <c r="E64" t="s">
         <v>38</v>
@@ -5363,9 +5670,9 @@
         <v>748</v>
       </c>
     </row>
-    <row r="65" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A65">
-        <v>12059099009</v>
+    <row r="65" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>361</v>
       </c>
       <c r="D65">
         <v>6155559</v>
@@ -5416,9 +5723,9 @@
         <v>793</v>
       </c>
     </row>
-    <row r="66" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A66">
-        <v>18604947620</v>
+    <row r="66" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>362</v>
       </c>
       <c r="E66" t="s">
         <v>38</v>
@@ -5469,9 +5776,9 @@
         <v>814</v>
       </c>
     </row>
-    <row r="67" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A67">
-        <v>14698088704</v>
+    <row r="67" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>363</v>
       </c>
       <c r="D67" t="s">
         <v>217</v>
@@ -5528,9 +5835,9 @@
         <v>817</v>
       </c>
     </row>
-    <row r="68" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A68">
-        <v>12122082849</v>
+    <row r="68" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>364</v>
       </c>
       <c r="E68" t="s">
         <v>38</v>
@@ -5581,9 +5888,9 @@
         <v>827</v>
       </c>
     </row>
-    <row r="69" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A69">
-        <v>18446210949</v>
+    <row r="69" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>365</v>
       </c>
       <c r="E69" t="s">
         <v>38</v>
@@ -5634,9 +5941,9 @@
         <v>856</v>
       </c>
     </row>
-    <row r="70" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A70">
-        <v>16038981747</v>
+    <row r="70" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>366</v>
       </c>
       <c r="E70" t="s">
         <v>38</v>
@@ -5687,9 +5994,9 @@
         <v>859</v>
       </c>
     </row>
-    <row r="71" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A71">
-        <v>12704186304</v>
+    <row r="71" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>367</v>
       </c>
       <c r="E71" t="s">
         <v>38</v>
@@ -5743,9 +6050,9 @@
         <v>869</v>
       </c>
     </row>
-    <row r="72" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A72">
-        <v>16094037594</v>
+    <row r="72" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>368</v>
       </c>
       <c r="D72">
         <v>6150394</v>
@@ -5796,9 +6103,9 @@
         <v>872</v>
       </c>
     </row>
-    <row r="73" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A73">
-        <v>18084870628</v>
+    <row r="73" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>369</v>
       </c>
       <c r="E73" t="s">
         <v>38</v>
@@ -5849,9 +6156,9 @@
         <v>887</v>
       </c>
     </row>
-    <row r="74" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A74">
-        <v>18005987561</v>
+    <row r="74" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>370</v>
       </c>
       <c r="E74" t="s">
         <v>38</v>
@@ -5902,9 +6209,9 @@
         <v>889</v>
       </c>
     </row>
-    <row r="75" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A75">
-        <v>18448591664</v>
+    <row r="75" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>371</v>
       </c>
       <c r="E75" t="s">
         <v>38</v>
@@ -5955,9 +6262,9 @@
         <v>901</v>
       </c>
     </row>
-    <row r="76" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A76">
-        <v>18442153023</v>
+    <row r="76" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>372</v>
       </c>
       <c r="E76" t="s">
         <v>38</v>
@@ -6008,9 +6315,9 @@
         <v>904</v>
       </c>
     </row>
-    <row r="77" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A77">
-        <v>17704072207</v>
+    <row r="77" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>373</v>
       </c>
       <c r="D77">
         <v>6190011</v>
@@ -6061,9 +6368,9 @@
         <v>917</v>
       </c>
     </row>
-    <row r="78" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A78">
-        <v>16237071176</v>
+    <row r="78" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>374</v>
       </c>
       <c r="D78" t="s">
         <v>244</v>
@@ -6120,9 +6427,9 @@
         <v>925</v>
       </c>
     </row>
-    <row r="79" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A79">
-        <v>11165122202</v>
+    <row r="79" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>375</v>
       </c>
       <c r="E79" t="s">
         <v>38</v>
@@ -6170,9 +6477,9 @@
         <v>934</v>
       </c>
     </row>
-    <row r="80" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A80">
-        <v>18447172505</v>
+    <row r="80" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>376</v>
       </c>
       <c r="E80" t="s">
         <v>38</v>
@@ -6223,9 +6530,9 @@
         <v>939</v>
       </c>
     </row>
-    <row r="81" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A81">
-        <v>16827858101</v>
+    <row r="81" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>377</v>
       </c>
       <c r="D81" t="s">
         <v>252</v>
@@ -6282,9 +6589,9 @@
         <v>951</v>
       </c>
     </row>
-    <row r="82" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A82">
-        <v>18452886684</v>
+    <row r="82" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>378</v>
       </c>
       <c r="D82">
         <v>6153449</v>
@@ -6335,9 +6642,9 @@
         <v>968</v>
       </c>
     </row>
-    <row r="83" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A83">
-        <v>19086731724</v>
+    <row r="83" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>379</v>
       </c>
       <c r="E83" t="s">
         <v>38</v>
@@ -6391,9 +6698,9 @@
         <v>972</v>
       </c>
     </row>
-    <row r="84" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A84">
-        <v>14072043651</v>
+    <row r="84" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>380</v>
       </c>
       <c r="E84" t="s">
         <v>38</v>
@@ -6447,9 +6754,9 @@
         <v>983</v>
       </c>
     </row>
-    <row r="85" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A85">
-        <v>11165122318</v>
+    <row r="85" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>381</v>
       </c>
       <c r="E85" t="s">
         <v>38</v>
@@ -6497,9 +6804,9 @@
         <v>986</v>
       </c>
     </row>
-    <row r="86" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A86">
-        <v>15086213800</v>
+    <row r="86" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>382</v>
       </c>
       <c r="E86" t="s">
         <v>38</v>
@@ -6553,9 +6860,9 @@
         <v>994</v>
       </c>
     </row>
-    <row r="87" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A87">
-        <v>12813924333</v>
+    <row r="87" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>383</v>
       </c>
       <c r="E87" t="s">
         <v>38</v>
@@ -6606,9 +6913,9 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="88" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A88">
-        <v>12038050236</v>
+    <row r="88" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>384</v>
       </c>
       <c r="E88" t="s">
         <v>38</v>
@@ -6662,9 +6969,9 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="89" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A89">
-        <v>12068920075</v>
+    <row r="89" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>385</v>
       </c>
       <c r="E89" t="s">
         <v>38</v>
@@ -6712,9 +7019,9 @@
         <v>1051</v>
       </c>
     </row>
-    <row r="90" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A90">
-        <v>19785393223</v>
+    <row r="90" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>386</v>
       </c>
       <c r="D90">
         <v>6150387</v>
@@ -6765,9 +7072,9 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="91" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A91">
-        <v>14402642930</v>
+    <row r="91" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>387</v>
       </c>
       <c r="E91" t="s">
         <v>38</v>
@@ -6821,9 +7128,9 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="92" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A92">
-        <v>17044965969</v>
+    <row r="92" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>388</v>
       </c>
       <c r="D92">
         <v>7157774</v>
@@ -6874,9 +7181,9 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="93" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A93">
-        <v>13035680570</v>
+    <row r="93" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>389</v>
       </c>
       <c r="D93" t="s">
         <v>277</v>
@@ -6933,9 +7240,9 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="94" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A94">
-        <v>18134396643</v>
+    <row r="94" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>390</v>
       </c>
       <c r="E94" t="s">
         <v>38</v>
@@ -6989,9 +7296,9 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="95" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A95">
-        <v>17192160070</v>
+    <row r="95" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>391</v>
       </c>
       <c r="D95" t="s">
         <v>283</v>
@@ -7048,9 +7355,9 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="96" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A96">
-        <v>16144582016</v>
+    <row r="96" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>392</v>
       </c>
       <c r="E96" t="s">
         <v>38</v>
@@ -7104,9 +7411,9 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="97" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A97">
-        <v>17029639622</v>
+    <row r="97" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>393</v>
       </c>
       <c r="D97" t="s">
         <v>290</v>
@@ -7163,9 +7470,9 @@
         <v>1106</v>
       </c>
     </row>
-    <row r="98" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A98">
-        <v>17043601846</v>
+    <row r="98" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>394</v>
       </c>
       <c r="E98" t="s">
         <v>38</v>
@@ -7219,9 +7526,9 @@
         <v>1113</v>
       </c>
     </row>
-    <row r="99" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A99">
-        <v>17815651907</v>
+    <row r="99" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>395</v>
       </c>
       <c r="D99">
         <v>6150331</v>

</xml_diff>